<commit_message>
Se actualiza Mapa de Sitios y se agrega guia de usuario para RNU
</commit_message>
<xml_diff>
--- a/Sitios MBB/Reemplazos a realizar en Sitios.xlsx
+++ b/Sitios MBB/Reemplazos a realizar en Sitios.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/69517450a5f14e94/Intranet/Sitios MBB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="292" documentId="8_{C5BAA5DA-583E-4BCA-9836-C3A43265B10E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D65713A1-4553-4B9F-931C-9C499240A2FA}"/>
+  <xr:revisionPtr revIDLastSave="303" documentId="8_{C5BAA5DA-583E-4BCA-9836-C3A43265B10E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A27429E3-748B-44E3-8DDB-1274ECDD5584}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{EF617B91-231F-446F-9C8D-9D09E3385D4E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="253">
   <si>
     <t>BUSCAR</t>
   </si>
@@ -533,9 +533,6 @@
     <t>Nochistlán de Mejía</t>
   </si>
   <si>
-    <t>San LuisPotosí</t>
-  </si>
-  <si>
     <t>San Felipe Orizatl�n</t>
   </si>
   <si>
@@ -768,6 +765,36 @@
   </si>
   <si>
     <t>Ixtlán del Río</t>
+  </si>
+  <si>
+    <t>UBICACI�N</t>
+  </si>
+  <si>
+    <t>Quer�taro</t>
+  </si>
+  <si>
+    <t>Michoac�n</t>
+  </si>
+  <si>
+    <t>San Luis Potos�</t>
+  </si>
+  <si>
+    <t>San Luis Potosí</t>
+  </si>
+  <si>
+    <t>Yucat�n</t>
+  </si>
+  <si>
+    <t>Coyoacan</t>
+  </si>
+  <si>
+    <t>Nezahualc�yotl</t>
+  </si>
+  <si>
+    <t>Alvaro Obregon</t>
+  </si>
+  <si>
+    <t>Naucalpan de Juarez</t>
   </si>
 </sst>
 </file>
@@ -869,17 +896,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1220,7 +1237,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5A7AFB2-C9AD-4CFE-B0B7-3A4601322FD3}">
-  <dimension ref="B2:D129"/>
+  <dimension ref="B2:D128"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="3" width="30.7109375" style="1" customWidth="1"/>
@@ -1238,46 +1255,73 @@
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="1" t="s">
+        <v>243</v>
+      </c>
       <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>244</v>
+      </c>
       <c r="C4" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
+        <v>245</v>
+      </c>
       <c r="C5" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
+        <v>246</v>
+      </c>
       <c r="C6" s="1" t="s">
-        <v>165</v>
+        <v>247</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
+        <v>248</v>
+      </c>
       <c r="C7" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="s">
+        <v>249</v>
+      </c>
       <c r="C8" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B9" s="1" t="s">
+        <v>250</v>
+      </c>
       <c r="C9" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
+        <v>251</v>
+      </c>
       <c r="C10" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
+        <v>252</v>
+      </c>
       <c r="C11" s="1" t="s">
         <v>9</v>
       </c>
@@ -1810,100 +1854,108 @@
         <v>144</v>
       </c>
     </row>
+    <row r="78" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B78" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>146</v>
+      </c>
+    </row>
     <row r="79" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B79" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="80" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B80" s="1" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="81" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B81" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="82" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B82" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="83" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B83" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="84" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B84" s="1" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="85" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B85" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="86" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B86" s="1" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="87" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B87" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="88" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B88" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="89" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B89" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="90" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B90" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>169</v>
+        <v>10</v>
       </c>
     </row>
     <row r="91" spans="2:3" x14ac:dyDescent="0.25">
@@ -1911,23 +1963,23 @@
         <v>170</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>10</v>
+        <v>171</v>
       </c>
     </row>
     <row r="92" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B92" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="93" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B93" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>174</v>
+        <v>11</v>
       </c>
     </row>
     <row r="94" spans="2:3" x14ac:dyDescent="0.25">
@@ -1935,52 +1987,52 @@
         <v>175</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>11</v>
+        <v>176</v>
       </c>
     </row>
     <row r="95" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B95" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="96" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B96" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="97" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B97" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="98" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B98" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="99" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B99" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="100" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B100" s="1" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C100" s="1" t="s">
         <v>187</v>
@@ -1991,44 +2043,44 @@
         <v>189</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="102" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B102" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="103" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B103" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="104" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B104" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="105" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B105" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="106" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B106" s="1" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>199</v>
@@ -2039,63 +2091,63 @@
         <v>201</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="108" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B108" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="109" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B109" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="110" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B110" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="111" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B111" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="112" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B112" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="113" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B113" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="114" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B114" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="115" spans="2:3" x14ac:dyDescent="0.25">
@@ -2108,7 +2160,7 @@
     </row>
     <row r="116" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B116" s="1" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>219</v>
@@ -2119,7 +2171,7 @@
         <v>221</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="118" spans="2:3" x14ac:dyDescent="0.25">
@@ -2132,95 +2184,87 @@
     </row>
     <row r="119" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B119" s="1" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="120" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B120" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="121" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B121" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="122" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B122" s="1" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
     </row>
     <row r="123" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B123" s="1" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
     </row>
     <row r="124" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B124" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="125" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B125" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="126" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B126" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="127" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B127" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="128" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B128" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="129" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B129" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="C129" s="1" t="s">
-        <v>243</v>
-      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C120:C197 C2:C15 C18:C114">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  <conditionalFormatting sqref="C119:C196 C2:C15 C18:C113">
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>